<commit_message>
Update led screen control
</commit_message>
<xml_diff>
--- a/Resources/MixerReportForm.xlsx
+++ b/Resources/MixerReportForm.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\TechlinkProjects\mixer-control-globalver\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F47AA0F4-15BF-4589-A607-928C4D2A1CA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4A68B73-D328-419A-A04C-B93DD5248487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{47E0C17C-C30F-4C83-B76F-2A7D44E858BA}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{47E0C17C-C30F-4C83-B76F-2A7D44E858BA}"/>
   </bookViews>
   <sheets>
     <sheet name="material_report" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t xml:space="preserve">MIXER REPORT - </t>
   </si>
@@ -118,6 +118,10 @@
   </si>
   <si>
     <t>Time end oil feed</t>
+  </si>
+  <si>
+    <t>Oil mass deviation
+(L)</t>
   </si>
 </sst>
 </file>
@@ -125,8 +129,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="166" formatCode="[$]dd/mm/yyyy;@" x16r2:formatCode16="[$-en-001,1]dd/mm/yyyy;@"/>
-    <numFmt numFmtId="168" formatCode="[$]hh:mm:ss;@" x16r2:formatCode16="[$-en-001,1]hh:mm:ss;@"/>
+    <numFmt numFmtId="164" formatCode="[$]dd/mm/yyyy;@" x16r2:formatCode16="[$-en-001,1]dd/mm/yyyy;@"/>
+    <numFmt numFmtId="165" formatCode="[$]hh:mm:ss;@" x16r2:formatCode16="[$-en-001,1]hh:mm:ss;@"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -286,9 +290,33 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -305,30 +333,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -645,7 +649,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E26985B9-2482-434E-9233-05467D2EA43F}">
-  <dimension ref="A1:U8"/>
+  <dimension ref="A1:V8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.6640625" style="1" customWidth="1"/>
@@ -654,53 +658,53 @@
     <col min="4" max="5" width="3.33203125" style="2" customWidth="1"/>
     <col min="6" max="6" width="11.6640625" style="1" customWidth="1"/>
     <col min="7" max="7" width="20.21875" style="9" customWidth="1"/>
-    <col min="8" max="8" width="17.33203125" style="27" customWidth="1"/>
-    <col min="9" max="9" width="18.77734375" style="28" customWidth="1"/>
-    <col min="10" max="10" width="20" style="24" customWidth="1"/>
-    <col min="11" max="11" width="20" style="28" customWidth="1"/>
+    <col min="8" max="8" width="17.33203125" style="20" customWidth="1"/>
+    <col min="9" max="9" width="18.77734375" style="21" customWidth="1"/>
+    <col min="10" max="10" width="20" style="17" customWidth="1"/>
+    <col min="11" max="11" width="20" style="21" customWidth="1"/>
     <col min="12" max="12" width="19.5546875" style="1" customWidth="1"/>
     <col min="13" max="14" width="17.21875" style="1" customWidth="1"/>
     <col min="15" max="15" width="21" style="1" customWidth="1"/>
-    <col min="16" max="16" width="19.5546875" style="24" customWidth="1"/>
-    <col min="17" max="17" width="18.6640625" style="28" customWidth="1"/>
-    <col min="18" max="18" width="19.77734375" style="24" customWidth="1"/>
-    <col min="19" max="19" width="17.5546875" style="28" customWidth="1"/>
+    <col min="16" max="16" width="19.5546875" style="17" customWidth="1"/>
+    <col min="17" max="17" width="18.6640625" style="21" customWidth="1"/>
+    <col min="18" max="18" width="19.77734375" style="17" customWidth="1"/>
+    <col min="19" max="19" width="17.5546875" style="21" customWidth="1"/>
     <col min="20" max="20" width="14.5546875" style="1" customWidth="1"/>
     <col min="21" max="21" width="18.109375" style="1" customWidth="1"/>
-    <col min="22" max="22" width="13.88671875" style="1" customWidth="1"/>
+    <col min="22" max="22" width="19.77734375" style="1" customWidth="1"/>
     <col min="23" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:22" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="19"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="27"/>
       <c r="M1" s="10"/>
       <c r="N1" s="10"/>
       <c r="O1" s="10"/>
     </row>
-    <row r="2" spans="1:21" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="26"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="19"/>
       <c r="I2" s="13" t="s">
         <v>12</v>
       </c>
@@ -715,17 +719,17 @@
       <c r="N2" s="11"/>
       <c r="O2" s="11"/>
     </row>
-    <row r="3" spans="1:21" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="26"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="19"/>
       <c r="I3" s="14"/>
       <c r="J3" s="14"/>
       <c r="K3" s="14"/>
@@ -734,36 +738,36 @@
       <c r="N3" s="12"/>
       <c r="O3" s="12"/>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
       <c r="J4" s="15"/>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
       <c r="J5" s="15"/>
     </row>
-    <row r="6" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="16" t="s">
+    <row r="6" spans="1:22" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="16"/>
+      <c r="B6" s="23"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
-      <c r="F6" s="16" t="s">
+      <c r="F6" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
-      <c r="I6" s="29"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="24"/>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="J7" s="15"/>
     </row>
-    <row r="8" spans="1:21" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>4</v>
       </c>
@@ -779,16 +783,16 @@
       <c r="G8" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="23" t="s">
+      <c r="H8" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="30" t="s">
+      <c r="I8" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="J8" s="23" t="s">
+      <c r="J8" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="K8" s="30" t="s">
+      <c r="K8" s="22" t="s">
         <v>21</v>
       </c>
       <c r="L8" s="6" t="s">
@@ -803,16 +807,16 @@
       <c r="O8" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="P8" s="23" t="s">
+      <c r="P8" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="Q8" s="30" t="s">
+      <c r="Q8" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="R8" s="23" t="s">
+      <c r="R8" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="S8" s="30" t="s">
+      <c r="S8" s="22" t="s">
         <v>26</v>
       </c>
       <c r="T8" s="6" t="s">
@@ -820,6 +824,9 @@
       </c>
       <c r="U8" s="6" t="s">
         <v>18</v>
+      </c>
+      <c r="V8" s="6" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>